<commit_message>
Add verified NABIL NPL and CAR data from annual reports
Cross-verified GNPL% from loan classification tables across 3 annual reports:
- FY2020: 0.74% (FY2023 report 5-yr summary + FY2025 report)
- FY2021: 0.84% (FY2023 report loan table + FY2025 report + ICRA)
- FY2022-2024: Updated to annual report GNPL (1.62%, 3.39%, 4.45%)
  replacing NRB supervision report values for consistent methodology
- FY2025: 4.48% (FY2025 report audited loan classification table)

CAR FY2025: 11.81% from FY2025 annual report CAR table (line 3719)

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/MASTER/master_bank_panel.xlsx
+++ b/MASTER/master_bank_panel.xlsx
@@ -18214,12 +18214,24 @@
       <c r="AJ68" t="n">
         <v>34.79023776487428</v>
       </c>
-      <c r="AK68" t="inlineStr"/>
-      <c r="AL68" t="inlineStr"/>
-      <c r="AM68" t="inlineStr"/>
-      <c r="AN68" t="inlineStr"/>
-      <c r="AO68" t="inlineStr"/>
-      <c r="AP68" t="inlineStr"/>
+      <c r="AK68" t="n">
+        <v>118.2692835820896</v>
+      </c>
+      <c r="AL68" t="n">
+        <v>73.74696019900499</v>
+      </c>
+      <c r="AM68" t="n">
+        <v>94.92859203980099</v>
+      </c>
+      <c r="AN68" t="n">
+        <v>1.723004975124378</v>
+      </c>
+      <c r="AO68" t="n">
+        <v>1997.657647058824</v>
+      </c>
+      <c r="AP68" t="n">
+        <v>0.74</v>
+      </c>
       <c r="AQ68" t="inlineStr"/>
       <c r="AR68" t="inlineStr"/>
       <c r="AS68" t="n">
@@ -18255,8 +18267,12 @@
       <c r="BC68" t="n">
         <v>2</v>
       </c>
-      <c r="BD68" t="inlineStr"/>
-      <c r="BE68" t="inlineStr"/>
+      <c r="BD68" t="n">
+        <v>119</v>
+      </c>
+      <c r="BE68" t="n">
+        <v>2010</v>
+      </c>
       <c r="BF68" t="inlineStr"/>
       <c r="BG68" t="inlineStr"/>
       <c r="BH68" t="inlineStr"/>
@@ -18490,12 +18506,24 @@
       <c r="AJ69" t="n">
         <v>9.029001728182235</v>
       </c>
-      <c r="AK69" t="inlineStr"/>
-      <c r="AL69" t="inlineStr"/>
-      <c r="AM69" t="inlineStr"/>
-      <c r="AN69" t="inlineStr"/>
-      <c r="AO69" t="inlineStr"/>
-      <c r="AP69" t="inlineStr"/>
+      <c r="AK69" t="n">
+        <v>134.3796029547553</v>
+      </c>
+      <c r="AL69" t="n">
+        <v>91.42263157894737</v>
+      </c>
+      <c r="AM69" t="n">
+        <v>103.1738088642659</v>
+      </c>
+      <c r="AN69" t="n">
+        <v>2.09028162511542</v>
+      </c>
+      <c r="AO69" t="n">
+        <v>2156.046074074074</v>
+      </c>
+      <c r="AP69" t="n">
+        <v>0.84</v>
+      </c>
       <c r="AQ69" t="inlineStr"/>
       <c r="AR69" t="inlineStr"/>
       <c r="AS69" t="n">
@@ -18531,8 +18559,12 @@
       <c r="BC69" t="n">
         <v>1</v>
       </c>
-      <c r="BD69" t="inlineStr"/>
-      <c r="BE69" t="inlineStr"/>
+      <c r="BD69" t="n">
+        <v>135</v>
+      </c>
+      <c r="BE69" t="n">
+        <v>2166</v>
+      </c>
       <c r="BF69" t="n">
         <v>148</v>
       </c>
@@ -18776,13 +18808,23 @@
       <c r="AJ70" t="n">
         <v>8.923427439844437</v>
       </c>
-      <c r="AK70" t="inlineStr"/>
-      <c r="AL70" t="inlineStr"/>
-      <c r="AM70" t="inlineStr"/>
-      <c r="AN70" t="inlineStr"/>
-      <c r="AO70" t="inlineStr"/>
+      <c r="AK70" t="n">
+        <v>187.8380760626398</v>
+      </c>
+      <c r="AL70" t="n">
+        <v>134.3202013422819</v>
+      </c>
+      <c r="AM70" t="n">
+        <v>145.9607651006712</v>
+      </c>
+      <c r="AN70" t="n">
+        <v>1.904259507829978</v>
+      </c>
+      <c r="AO70" t="n">
+        <v>1817.394372294372</v>
+      </c>
       <c r="AP70" t="n">
-        <v>4.5</v>
+        <v>1.62</v>
       </c>
       <c r="AQ70" t="n">
         <v>2.02</v>
@@ -18823,8 +18865,12 @@
       <c r="BC70" t="n">
         <v>3</v>
       </c>
-      <c r="BD70" t="inlineStr"/>
-      <c r="BE70" t="inlineStr"/>
+      <c r="BD70" t="n">
+        <v>231</v>
+      </c>
+      <c r="BE70" t="n">
+        <v>2235</v>
+      </c>
       <c r="BF70" t="n">
         <v>163</v>
       </c>
@@ -19066,13 +19112,23 @@
       <c r="AJ71" t="n">
         <v>7.111801675652793</v>
       </c>
-      <c r="AK71" t="inlineStr"/>
-      <c r="AL71" t="inlineStr"/>
-      <c r="AM71" t="inlineStr"/>
-      <c r="AN71" t="inlineStr"/>
-      <c r="AO71" t="inlineStr"/>
+      <c r="AK71" t="n">
+        <v>200.1678660565724</v>
+      </c>
+      <c r="AL71" t="n">
+        <v>137.7384234608985</v>
+      </c>
+      <c r="AM71" t="n">
+        <v>165.0763311148087</v>
+      </c>
+      <c r="AN71" t="n">
+        <v>2.664284525790349</v>
+      </c>
+      <c r="AO71" t="n">
+        <v>1956.111991869919</v>
+      </c>
       <c r="AP71" t="n">
-        <v>3.99</v>
+        <v>3.39</v>
       </c>
       <c r="AQ71" t="n">
         <v>1.8</v>
@@ -19113,8 +19169,12 @@
       <c r="BC71" t="n">
         <v>2</v>
       </c>
-      <c r="BD71" t="inlineStr"/>
-      <c r="BE71" t="inlineStr"/>
+      <c r="BD71" t="n">
+        <v>246</v>
+      </c>
+      <c r="BE71" t="n">
+        <v>2404</v>
+      </c>
       <c r="BF71" t="n">
         <v>223</v>
       </c>
@@ -19356,13 +19416,23 @@
       <c r="AJ72" t="n">
         <v>8.297967245915586</v>
       </c>
-      <c r="AK72" t="inlineStr"/>
-      <c r="AL72" t="inlineStr"/>
-      <c r="AM72" t="inlineStr"/>
-      <c r="AN72" t="inlineStr"/>
-      <c r="AO72" t="inlineStr"/>
+      <c r="AK72" t="n">
+        <v>231.7054450915142</v>
+      </c>
+      <c r="AL72" t="n">
+        <v>160.4509567387687</v>
+      </c>
+      <c r="AM72" t="n">
+        <v>192.220224625624</v>
+      </c>
+      <c r="AN72" t="n">
+        <v>2.577832778702163</v>
+      </c>
+      <c r="AO72" t="n">
+        <v>2094.059736842105</v>
+      </c>
       <c r="AP72" t="n">
-        <v>3.6</v>
+        <v>4.45</v>
       </c>
       <c r="AQ72" t="n">
         <v>1.62</v>
@@ -19403,8 +19473,12 @@
       <c r="BC72" t="n">
         <v>1</v>
       </c>
-      <c r="BD72" t="inlineStr"/>
-      <c r="BE72" t="inlineStr"/>
+      <c r="BD72" t="n">
+        <v>266</v>
+      </c>
+      <c r="BE72" t="n">
+        <v>2404</v>
+      </c>
       <c r="BF72" t="n">
         <v>240</v>
       </c>
@@ -19660,15 +19734,29 @@
       <c r="AJ73" t="n">
         <v>8.378398964125218</v>
       </c>
-      <c r="AK73" t="inlineStr"/>
-      <c r="AL73" t="inlineStr"/>
-      <c r="AM73" t="inlineStr"/>
-      <c r="AN73" t="inlineStr"/>
-      <c r="AO73" t="inlineStr"/>
-      <c r="AP73" t="inlineStr"/>
+      <c r="AK73" t="n">
+        <v>265.1071482098251</v>
+      </c>
+      <c r="AL73" t="n">
+        <v>171.1040965861782</v>
+      </c>
+      <c r="AM73" t="n">
+        <v>218.4121398834305</v>
+      </c>
+      <c r="AN73" t="n">
+        <v>2.465503746877602</v>
+      </c>
+      <c r="AO73" t="n">
+        <v>2376.072276119403</v>
+      </c>
+      <c r="AP73" t="n">
+        <v>4.48</v>
+      </c>
       <c r="AQ73" t="inlineStr"/>
       <c r="AR73" t="inlineStr"/>
-      <c r="AS73" t="inlineStr"/>
+      <c r="AS73" t="n">
+        <v>11.81</v>
+      </c>
       <c r="AT73" t="inlineStr"/>
       <c r="AU73" t="n">
         <v>78.34001199635642</v>
@@ -19697,8 +19785,12 @@
       <c r="BC73" t="n">
         <v>1</v>
       </c>
-      <c r="BD73" t="inlineStr"/>
-      <c r="BE73" t="inlineStr"/>
+      <c r="BD73" t="n">
+        <v>268</v>
+      </c>
+      <c r="BE73" t="n">
+        <v>2402</v>
+      </c>
       <c r="BF73" t="n">
         <v>244</v>
       </c>
@@ -39423,10 +39515,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="39">
@@ -39436,10 +39528,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="40">
@@ -39449,10 +39541,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="41">
@@ -39462,10 +39554,10 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="42">
@@ -39475,10 +39567,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C42" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="43">
@@ -39488,10 +39580,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C43" t="n">
-        <v>43.5</v>
+        <v>45.7</v>
       </c>
     </row>
     <row r="44">
@@ -39527,10 +39619,10 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C46" t="n">
-        <v>76.8</v>
+        <v>77.5</v>
       </c>
     </row>
     <row r="47">
@@ -39670,10 +39762,10 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C57" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="58">
@@ -39683,10 +39775,10 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C58" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="59">

</xml_diff>